<commit_message>
Add Guardant Health to the Summary sheet of the model workbook
GH (Buy, high risk; ~$150 base target) now appears in the four-name ratings
table with a source link; note points to GuardantHealthAnalysis.md for the
full GH model.

https://claude.ai/code/session_01GzmMSx9zTnCS3tbwnbT4wp
</commit_message>
<xml_diff>
--- a/StockAnalysis.xlsx
+++ b/StockAnalysis.xlsx
@@ -499,10 +499,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -522,7 +522,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Educational exercise; NOT investment advice. Figures from public sources as of late May 2026. 'E' = illustrative analyst estimate.</t>
+          <t>Educational exercise; NOT investment advice. Figures from public sources as of late May 2026. 'E' = illustrative estimate. Detail sheets cover Amgen/Danaher/Sandoz; the full Guardant Health model lives in GuardantHealthAnalysis.md.</t>
         </is>
       </c>
     </row>
@@ -691,6 +691,48 @@
       <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Investing.com - Sandoz price/market data</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Guardant Health</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>GH (Nasdaq)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Liquid-biopsy diagnostics</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>~$127</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>BUY (high risk)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>~$150</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>~+18% (no dividend)</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>stockanalysis.com - GH statistics</t>
         </is>
       </c>
     </row>
@@ -699,6 +741,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1102,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1348,6 +1391,21 @@
       <c r="C18" s="6" t="inlineStr">
         <is>
           <t>https://www.investing.com/equities/sandoz</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>stockanalysis.com - GH statistics</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>https://stockanalysis.com/stocks/gh/</t>
         </is>
       </c>
     </row>
@@ -1367,6 +1425,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>